<commit_message>
todos, Take On Me: alte Kalkulations-/Tabellenreste entfernt, Tabelle aktualisiert
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/TakeOnMe_v1/quelle/struktur.xlsx
+++ b/songs/TakeOnMe_v1/quelle/struktur.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\00_DATEN\PlatformIO\Projects\LED-GIT_on_YULC\songs\TakeOnMe_v1\quelle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D71D9C5-C07A-479C-A2FF-DF80D5874F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{620F14DC-6460-482F-B3D0-A80E8F3D7DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36" yWindow="888" windowWidth="31908" windowHeight="24192" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7536" yWindow="2820" windowWidth="38352" windowHeight="20436" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Struktur" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="93">
   <si>
     <t>Take On Me</t>
   </si>
@@ -394,12 +394,6 @@
   </si>
   <si>
     <t>10 sek. BLACK</t>
-  </si>
-  <si>
-    <t>das letzte take on me scheint noch zu fehlen …irgendwas ist hier noch nicht so wie oben ab 44 und 80!</t>
-  </si>
-  <si>
-    <t>die schwarz ausgestanzte rund um die schrift erkennt man nur beim letzten me …warum auch immer !?</t>
   </si>
 </sst>
 </file>
@@ -2838,9 +2832,7 @@
       <c r="C166" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D166" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="D166" s="8"/>
       <c r="E166" s="6"/>
       <c r="F166" s="5"/>
       <c r="G166" s="5">
@@ -7398,9 +7390,7 @@
       <c r="C534" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D534" s="8" t="s">
-        <v>93</v>
-      </c>
+      <c r="D534" s="8"/>
       <c r="E534" s="6"/>
       <c r="F534" s="5"/>
       <c r="G534" s="5">

</xml_diff>